<commit_message>
Make CodeGen QUESTIONS[] formulas live from the score grid.
Regenerate the workbook and document language pin software remap plus
clear-Artwork workflow so score and screen edits propagate on recalc.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/questions/MediaMap_workbook.xlsx
+++ b/questions/MediaMap_workbook.xlsx
@@ -578,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -700,109 +700,116 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Step number updates automatically. Copy dropdowns from the row above if needed.</t>
+          <t xml:space="preserve">  Clear Artwork to remove a step (do not delete rows — CodeGen uses fixed row refs).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Then copy CodeGen column A into QuestionnaireConfig.h (NUM_QUESTIONS + QUESTIONS[]).</t>
+          <t xml:space="preserve">  CodeGen column A updates when you edit scores, screen, or Artwork (recalc in Excel).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Or run: python scripts/generate_media_workbook.py --emit-cpp</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  SD WIZ1 / SD WIZ2 update automatically from Questions (clear Artwork to remove a step).</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>Sheets: Questions | SD WIZ1 | SD WIZ2 | CodeGen</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr"/>
-    </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>If CodeGen shows Err:508 in LibreOffice, run: python scripts/generate_media_workbook.py --emit-cpp</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="n"/>
-    </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="2" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Firmware limits</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Files per language (question text)</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>32</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Languages</t>
+          <t>Files per language (question text)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>32</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Max files per SD card</t>
+          <t>Languages</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Question rows in workbook</t>
+          <t>Max files per SD card</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>200</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>Question rows in workbook</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Quiz steps (initial)</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>13</t>
         </is>
@@ -810,7 +817,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="25">
+  <mergeCells count="26">
     <mergeCell ref="A5:D5"/>
     <mergeCell ref="A17:D17"/>
     <mergeCell ref="A23:D23"/>
@@ -831,6 +838,7 @@
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="A16:D16"/>
     <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A27:D27"/>
     <mergeCell ref="A12:D12"/>
     <mergeCell ref="A3:D3"/>
     <mergeCell ref="A21:D21"/>
@@ -1127,10 +1135,9 @@
       <c r="AB4" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="AC4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 1, Landscape, { { 10, 0, 0, 0 }, { 0, 10, 0, 0 }, { 0, 0, 10, 0 }, { 0, 0, 0, 10 } } },</t>
-        </is>
+      <c r="AC4">
+        <f>IF(B4="","","  { "&amp;E4&amp;", "&amp;IF(C4="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M4&amp;", "&amp;N4&amp;", "&amp;O4&amp;", "&amp;P4&amp;" }"&amp;", "&amp;" { "&amp;Q4&amp;", "&amp;R4&amp;", "&amp;S4&amp;", "&amp;T4&amp;" }"&amp;", "&amp;" { "&amp;U4&amp;", "&amp;V4&amp;", "&amp;W4&amp;", "&amp;X4&amp;" }"&amp;", "&amp;" { "&amp;Y4&amp;", "&amp;Z4&amp;", "&amp;AA4&amp;", "&amp;AB4&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -1232,10 +1239,9 @@
       <c r="AB5" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="AC5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 2, Portrait, { { 0, 0, 0, 10 }, { 0, 10, 0, 0 }, { 0, 0, 10, 0 }, { 10, 0, 0, 0 } } },</t>
-        </is>
+      <c r="AC5">
+        <f>IF(B5="","","  { "&amp;E5&amp;", "&amp;IF(C5="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M5&amp;", "&amp;N5&amp;", "&amp;O5&amp;", "&amp;P5&amp;" }"&amp;", "&amp;" { "&amp;Q5&amp;", "&amp;R5&amp;", "&amp;S5&amp;", "&amp;T5&amp;" }"&amp;", "&amp;" { "&amp;U5&amp;", "&amp;V5&amp;", "&amp;W5&amp;", "&amp;X5&amp;" }"&amp;", "&amp;" { "&amp;Y5&amp;", "&amp;Z5&amp;", "&amp;AA5&amp;", "&amp;AB5&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -1337,10 +1343,9 @@
       <c r="AB6" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="AC6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 3, Portrait, { { 10, 0, 0, 0 }, { 0, 10, 0, 0 }, { 0, 0, 10, 0 }, { 0, 0, 0, 10 } } },</t>
-        </is>
+      <c r="AC6">
+        <f>IF(B6="","","  { "&amp;E6&amp;", "&amp;IF(C6="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M6&amp;", "&amp;N6&amp;", "&amp;O6&amp;", "&amp;P6&amp;" }"&amp;", "&amp;" { "&amp;Q6&amp;", "&amp;R6&amp;", "&amp;S6&amp;", "&amp;T6&amp;" }"&amp;", "&amp;" { "&amp;U6&amp;", "&amp;V6&amp;", "&amp;W6&amp;", "&amp;X6&amp;" }"&amp;", "&amp;" { "&amp;Y6&amp;", "&amp;Z6&amp;", "&amp;AA6&amp;", "&amp;AB6&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -1442,10 +1447,9 @@
       <c r="AB7" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 4, Landscape, { { 10, 0, 0, 0 }, { 0, 10, 0, 0 }, { 0, 0, 10, 0 }, { 0, 0, 0, 10 } } },</t>
-        </is>
+      <c r="AC7">
+        <f>IF(B7="","","  { "&amp;E7&amp;", "&amp;IF(C7="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M7&amp;", "&amp;N7&amp;", "&amp;O7&amp;", "&amp;P7&amp;" }"&amp;", "&amp;" { "&amp;Q7&amp;", "&amp;R7&amp;", "&amp;S7&amp;", "&amp;T7&amp;" }"&amp;", "&amp;" { "&amp;U7&amp;", "&amp;V7&amp;", "&amp;W7&amp;", "&amp;X7&amp;" }"&amp;", "&amp;" { "&amp;Y7&amp;", "&amp;Z7&amp;", "&amp;AA7&amp;", "&amp;AB7&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -1547,10 +1551,9 @@
       <c r="AB8" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="AC8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 5, Landscape, { { 10, 0, 0, 0 }, { 0, 10, 0, 0 }, { 0, 0, 10, 0 }, { 0, 0, 0, 10 } } },</t>
-        </is>
+      <c r="AC8">
+        <f>IF(B8="","","  { "&amp;E8&amp;", "&amp;IF(C8="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M8&amp;", "&amp;N8&amp;", "&amp;O8&amp;", "&amp;P8&amp;" }"&amp;", "&amp;" { "&amp;Q8&amp;", "&amp;R8&amp;", "&amp;S8&amp;", "&amp;T8&amp;" }"&amp;", "&amp;" { "&amp;U8&amp;", "&amp;V8&amp;", "&amp;W8&amp;", "&amp;X8&amp;" }"&amp;", "&amp;" { "&amp;Y8&amp;", "&amp;Z8&amp;", "&amp;AA8&amp;", "&amp;AB8&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -1652,10 +1655,9 @@
       <c r="AB9" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 6, Landscape, { { 10, 0, 0, 0 }, { 0, 0, 0, 10 }, { 0, 0, 10, 0 }, { 0, 10, 0, 0 } } },</t>
-        </is>
+      <c r="AC9">
+        <f>IF(B9="","","  { "&amp;E9&amp;", "&amp;IF(C9="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M9&amp;", "&amp;N9&amp;", "&amp;O9&amp;", "&amp;P9&amp;" }"&amp;", "&amp;" { "&amp;Q9&amp;", "&amp;R9&amp;", "&amp;S9&amp;", "&amp;T9&amp;" }"&amp;", "&amp;" { "&amp;U9&amp;", "&amp;V9&amp;", "&amp;W9&amp;", "&amp;X9&amp;" }"&amp;", "&amp;" { "&amp;Y9&amp;", "&amp;Z9&amp;", "&amp;AA9&amp;", "&amp;AB9&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -1757,10 +1759,9 @@
       <c r="AB10" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="AC10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 7, Landscape, { { 0, 10, 0, 0 }, { 0, 0, 10, 0 }, { 0, 0, 0, 10 }, { 10, 0, 0, 0 } } },</t>
-        </is>
+      <c r="AC10">
+        <f>IF(B10="","","  { "&amp;E10&amp;", "&amp;IF(C10="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M10&amp;", "&amp;N10&amp;", "&amp;O10&amp;", "&amp;P10&amp;" }"&amp;", "&amp;" { "&amp;Q10&amp;", "&amp;R10&amp;", "&amp;S10&amp;", "&amp;T10&amp;" }"&amp;", "&amp;" { "&amp;U10&amp;", "&amp;V10&amp;", "&amp;W10&amp;", "&amp;X10&amp;" }"&amp;", "&amp;" { "&amp;Y10&amp;", "&amp;Z10&amp;", "&amp;AA10&amp;", "&amp;AB10&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -1862,10 +1863,9 @@
       <c r="AB11" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="AC11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 8, Portrait, { { 0, 0, 10, 0 }, { 0, 0, 0, 10 }, { 0, 10, 0, 0 }, { 10, 0, 0, 0 } } },</t>
-        </is>
+      <c r="AC11">
+        <f>IF(B11="","","  { "&amp;E11&amp;", "&amp;IF(C11="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M11&amp;", "&amp;N11&amp;", "&amp;O11&amp;", "&amp;P11&amp;" }"&amp;", "&amp;" { "&amp;Q11&amp;", "&amp;R11&amp;", "&amp;S11&amp;", "&amp;T11&amp;" }"&amp;", "&amp;" { "&amp;U11&amp;", "&amp;V11&amp;", "&amp;W11&amp;", "&amp;X11&amp;" }"&amp;", "&amp;" { "&amp;Y11&amp;", "&amp;Z11&amp;", "&amp;AA11&amp;", "&amp;AB11&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -1967,10 +1967,9 @@
       <c r="AB12" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 9, Landscape, { { 10, 0, 0, 0 }, { 0, 0, 0, 10 }, { 0, 10, 0, 0 }, { 0, 0, 10, 0 } } },</t>
-        </is>
+      <c r="AC12">
+        <f>IF(B12="","","  { "&amp;E12&amp;", "&amp;IF(C12="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M12&amp;", "&amp;N12&amp;", "&amp;O12&amp;", "&amp;P12&amp;" }"&amp;", "&amp;" { "&amp;Q12&amp;", "&amp;R12&amp;", "&amp;S12&amp;", "&amp;T12&amp;" }"&amp;", "&amp;" { "&amp;U12&amp;", "&amp;V12&amp;", "&amp;W12&amp;", "&amp;X12&amp;" }"&amp;", "&amp;" { "&amp;Y12&amp;", "&amp;Z12&amp;", "&amp;AA12&amp;", "&amp;AB12&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -2072,10 +2071,9 @@
       <c r="AB13" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="AC13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 10, Landscape, { { 0, 0, 10, 0 }, { 0, 0, 0, 10 }, { 0, 10, 0, 0 }, { 10, 0, 0, 0 } } },</t>
-        </is>
+      <c r="AC13">
+        <f>IF(B13="","","  { "&amp;E13&amp;", "&amp;IF(C13="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M13&amp;", "&amp;N13&amp;", "&amp;O13&amp;", "&amp;P13&amp;" }"&amp;", "&amp;" { "&amp;Q13&amp;", "&amp;R13&amp;", "&amp;S13&amp;", "&amp;T13&amp;" }"&amp;", "&amp;" { "&amp;U13&amp;", "&amp;V13&amp;", "&amp;W13&amp;", "&amp;X13&amp;" }"&amp;", "&amp;" { "&amp;Y13&amp;", "&amp;Z13&amp;", "&amp;AA13&amp;", "&amp;AB13&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="14">
@@ -2177,10 +2175,9 @@
       <c r="AB14" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="AC14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 11, Portrait, { { 10, 0, 0, 0 }, { 0, 0, 0, 10 }, { 0, 10, 0, 0 }, { 0, 0, 10, 0 } } },</t>
-        </is>
+      <c r="AC14">
+        <f>IF(B14="","","  { "&amp;E14&amp;", "&amp;IF(C14="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M14&amp;", "&amp;N14&amp;", "&amp;O14&amp;", "&amp;P14&amp;" }"&amp;", "&amp;" { "&amp;Q14&amp;", "&amp;R14&amp;", "&amp;S14&amp;", "&amp;T14&amp;" }"&amp;", "&amp;" { "&amp;U14&amp;", "&amp;V14&amp;", "&amp;W14&amp;", "&amp;X14&amp;" }"&amp;", "&amp;" { "&amp;Y14&amp;", "&amp;Z14&amp;", "&amp;AA14&amp;", "&amp;AB14&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
@@ -2282,10 +2279,9 @@
       <c r="AB15" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="AC15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 12, Landscape, { { 0, 10, 0, 0 }, { 10, 0, 0, 0 }, { 0, 0, 10, 0 }, { 0, 0, 0, 10 } } },</t>
-        </is>
+      <c r="AC15">
+        <f>IF(B15="","","  { "&amp;E15&amp;", "&amp;IF(C15="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M15&amp;", "&amp;N15&amp;", "&amp;O15&amp;", "&amp;P15&amp;" }"&amp;", "&amp;" { "&amp;Q15&amp;", "&amp;R15&amp;", "&amp;S15&amp;", "&amp;T15&amp;" }"&amp;", "&amp;" { "&amp;U15&amp;", "&amp;V15&amp;", "&amp;W15&amp;", "&amp;X15&amp;" }"&amp;", "&amp;" { "&amp;Y15&amp;", "&amp;Z15&amp;", "&amp;AA15&amp;", "&amp;AB15&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="16">
@@ -2387,10 +2383,9 @@
       <c r="AB16" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="AC16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  { 13, Portrait, { { 10, 0, 0, 0 }, { 0, 0, 0, 10 }, { 0, 10, 0, 0 }, { 0, 0, 10, 0 } } },</t>
-        </is>
+      <c r="AC16">
+        <f>IF(B16="","","  { "&amp;E16&amp;", "&amp;IF(C16="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M16&amp;", "&amp;N16&amp;", "&amp;O16&amp;", "&amp;P16&amp;" }"&amp;", "&amp;" { "&amp;Q16&amp;", "&amp;R16&amp;", "&amp;S16&amp;", "&amp;T16&amp;" }"&amp;", "&amp;" { "&amp;U16&amp;", "&amp;V16&amp;", "&amp;W16&amp;", "&amp;X16&amp;" }"&amp;", "&amp;" { "&amp;Y16&amp;", "&amp;Z16&amp;", "&amp;AA16&amp;", "&amp;AB16&amp;" }"&amp;" }"&amp;" } },")</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -2457,7 +2452,7 @@
       <c r="AA17" s="17" t="n"/>
       <c r="AB17" s="17" t="n"/>
       <c r="AC17">
-        <f>IF(B17="","","")</f>
+        <f>IF(B17="","","  { "&amp;E17&amp;", "&amp;IF(C17="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M17&amp;", "&amp;N17&amp;", "&amp;O17&amp;", "&amp;P17&amp;" }"&amp;", "&amp;" { "&amp;Q17&amp;", "&amp;R17&amp;", "&amp;S17&amp;", "&amp;T17&amp;" }"&amp;", "&amp;" { "&amp;U17&amp;", "&amp;V17&amp;", "&amp;W17&amp;", "&amp;X17&amp;" }"&amp;", "&amp;" { "&amp;Y17&amp;", "&amp;Z17&amp;", "&amp;AA17&amp;", "&amp;AB17&amp;" }"&amp;" }"&amp;" } },")</f>
         <v/>
       </c>
     </row>
@@ -2525,7 +2520,7 @@
       <c r="AA18" s="17" t="n"/>
       <c r="AB18" s="17" t="n"/>
       <c r="AC18">
-        <f>IF(B18="","","")</f>
+        <f>IF(B18="","","  { "&amp;E18&amp;", "&amp;IF(C18="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M18&amp;", "&amp;N18&amp;", "&amp;O18&amp;", "&amp;P18&amp;" }"&amp;", "&amp;" { "&amp;Q18&amp;", "&amp;R18&amp;", "&amp;S18&amp;", "&amp;T18&amp;" }"&amp;", "&amp;" { "&amp;U18&amp;", "&amp;V18&amp;", "&amp;W18&amp;", "&amp;X18&amp;" }"&amp;", "&amp;" { "&amp;Y18&amp;", "&amp;Z18&amp;", "&amp;AA18&amp;", "&amp;AB18&amp;" }"&amp;" }"&amp;" } },")</f>
         <v/>
       </c>
     </row>
@@ -2593,7 +2588,7 @@
       <c r="AA19" s="17" t="n"/>
       <c r="AB19" s="17" t="n"/>
       <c r="AC19">
-        <f>IF(B19="","","")</f>
+        <f>IF(B19="","","  { "&amp;E19&amp;", "&amp;IF(C19="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M19&amp;", "&amp;N19&amp;", "&amp;O19&amp;", "&amp;P19&amp;" }"&amp;", "&amp;" { "&amp;Q19&amp;", "&amp;R19&amp;", "&amp;S19&amp;", "&amp;T19&amp;" }"&amp;", "&amp;" { "&amp;U19&amp;", "&amp;V19&amp;", "&amp;W19&amp;", "&amp;X19&amp;" }"&amp;", "&amp;" { "&amp;Y19&amp;", "&amp;Z19&amp;", "&amp;AA19&amp;", "&amp;AB19&amp;" }"&amp;" }"&amp;" } },")</f>
         <v/>
       </c>
     </row>
@@ -2661,7 +2656,7 @@
       <c r="AA20" s="17" t="n"/>
       <c r="AB20" s="17" t="n"/>
       <c r="AC20">
-        <f>IF(B20="","","")</f>
+        <f>IF(B20="","","  { "&amp;E20&amp;", "&amp;IF(C20="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M20&amp;", "&amp;N20&amp;", "&amp;O20&amp;", "&amp;P20&amp;" }"&amp;", "&amp;" { "&amp;Q20&amp;", "&amp;R20&amp;", "&amp;S20&amp;", "&amp;T20&amp;" }"&amp;", "&amp;" { "&amp;U20&amp;", "&amp;V20&amp;", "&amp;W20&amp;", "&amp;X20&amp;" }"&amp;", "&amp;" { "&amp;Y20&amp;", "&amp;Z20&amp;", "&amp;AA20&amp;", "&amp;AB20&amp;" }"&amp;" }"&amp;" } },")</f>
         <v/>
       </c>
     </row>
@@ -2729,7 +2724,7 @@
       <c r="AA21" s="17" t="n"/>
       <c r="AB21" s="17" t="n"/>
       <c r="AC21">
-        <f>IF(B21="","","")</f>
+        <f>IF(B21="","","  { "&amp;E21&amp;", "&amp;IF(C21="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M21&amp;", "&amp;N21&amp;", "&amp;O21&amp;", "&amp;P21&amp;" }"&amp;", "&amp;" { "&amp;Q21&amp;", "&amp;R21&amp;", "&amp;S21&amp;", "&amp;T21&amp;" }"&amp;", "&amp;" { "&amp;U21&amp;", "&amp;V21&amp;", "&amp;W21&amp;", "&amp;X21&amp;" }"&amp;", "&amp;" { "&amp;Y21&amp;", "&amp;Z21&amp;", "&amp;AA21&amp;", "&amp;AB21&amp;" }"&amp;" }"&amp;" } },")</f>
         <v/>
       </c>
     </row>
@@ -2797,7 +2792,7 @@
       <c r="AA22" s="17" t="n"/>
       <c r="AB22" s="17" t="n"/>
       <c r="AC22">
-        <f>IF(B22="","","")</f>
+        <f>IF(B22="","","  { "&amp;E22&amp;", "&amp;IF(C22="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M22&amp;", "&amp;N22&amp;", "&amp;O22&amp;", "&amp;P22&amp;" }"&amp;", "&amp;" { "&amp;Q22&amp;", "&amp;R22&amp;", "&amp;S22&amp;", "&amp;T22&amp;" }"&amp;", "&amp;" { "&amp;U22&amp;", "&amp;V22&amp;", "&amp;W22&amp;", "&amp;X22&amp;" }"&amp;", "&amp;" { "&amp;Y22&amp;", "&amp;Z22&amp;", "&amp;AA22&amp;", "&amp;AB22&amp;" }"&amp;" }"&amp;" } },")</f>
         <v/>
       </c>
     </row>
@@ -2865,7 +2860,7 @@
       <c r="AA23" s="17" t="n"/>
       <c r="AB23" s="17" t="n"/>
       <c r="AC23">
-        <f>IF(B23="","","")</f>
+        <f>IF(B23="","","  { "&amp;E23&amp;", "&amp;IF(C23="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M23&amp;", "&amp;N23&amp;", "&amp;O23&amp;", "&amp;P23&amp;" }"&amp;", "&amp;" { "&amp;Q23&amp;", "&amp;R23&amp;", "&amp;S23&amp;", "&amp;T23&amp;" }"&amp;", "&amp;" { "&amp;U23&amp;", "&amp;V23&amp;", "&amp;W23&amp;", "&amp;X23&amp;" }"&amp;", "&amp;" { "&amp;Y23&amp;", "&amp;Z23&amp;", "&amp;AA23&amp;", "&amp;AB23&amp;" }"&amp;" }"&amp;" } },")</f>
         <v/>
       </c>
     </row>
@@ -2933,7 +2928,7 @@
       <c r="AA24" s="17" t="n"/>
       <c r="AB24" s="17" t="n"/>
       <c r="AC24">
-        <f>IF(B24="","","")</f>
+        <f>IF(B24="","","  { "&amp;E24&amp;", "&amp;IF(C24="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M24&amp;", "&amp;N24&amp;", "&amp;O24&amp;", "&amp;P24&amp;" }"&amp;", "&amp;" { "&amp;Q24&amp;", "&amp;R24&amp;", "&amp;S24&amp;", "&amp;T24&amp;" }"&amp;", "&amp;" { "&amp;U24&amp;", "&amp;V24&amp;", "&amp;W24&amp;", "&amp;X24&amp;" }"&amp;", "&amp;" { "&amp;Y24&amp;", "&amp;Z24&amp;", "&amp;AA24&amp;", "&amp;AB24&amp;" }"&amp;" }"&amp;" } },")</f>
         <v/>
       </c>
     </row>
@@ -3001,7 +2996,7 @@
       <c r="AA25" s="17" t="n"/>
       <c r="AB25" s="17" t="n"/>
       <c r="AC25">
-        <f>IF(B25="","","")</f>
+        <f>IF(B25="","","  { "&amp;E25&amp;", "&amp;IF(C25="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M25&amp;", "&amp;N25&amp;", "&amp;O25&amp;", "&amp;P25&amp;" }"&amp;", "&amp;" { "&amp;Q25&amp;", "&amp;R25&amp;", "&amp;S25&amp;", "&amp;T25&amp;" }"&amp;", "&amp;" { "&amp;U25&amp;", "&amp;V25&amp;", "&amp;W25&amp;", "&amp;X25&amp;" }"&amp;", "&amp;" { "&amp;Y25&amp;", "&amp;Z25&amp;", "&amp;AA25&amp;", "&amp;AB25&amp;" }"&amp;" }"&amp;" } },")</f>
         <v/>
       </c>
     </row>
@@ -3069,7 +3064,7 @@
       <c r="AA26" s="17" t="n"/>
       <c r="AB26" s="17" t="n"/>
       <c r="AC26">
-        <f>IF(B26="","","")</f>
+        <f>IF(B26="","","  { "&amp;E26&amp;", "&amp;IF(C26="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M26&amp;", "&amp;N26&amp;", "&amp;O26&amp;", "&amp;P26&amp;" }"&amp;", "&amp;" { "&amp;Q26&amp;", "&amp;R26&amp;", "&amp;S26&amp;", "&amp;T26&amp;" }"&amp;", "&amp;" { "&amp;U26&amp;", "&amp;V26&amp;", "&amp;W26&amp;", "&amp;X26&amp;" }"&amp;", "&amp;" { "&amp;Y26&amp;", "&amp;Z26&amp;", "&amp;AA26&amp;", "&amp;AB26&amp;" }"&amp;" }"&amp;" } },")</f>
         <v/>
       </c>
     </row>
@@ -3137,7 +3132,7 @@
       <c r="AA27" s="17" t="n"/>
       <c r="AB27" s="17" t="n"/>
       <c r="AC27">
-        <f>IF(B27="","","")</f>
+        <f>IF(B27="","","  { "&amp;E27&amp;", "&amp;IF(C27="Portrait","Portrait","Landscape")&amp;", "&amp;"{ "&amp;" { "&amp;M27&amp;", "&amp;N27&amp;", "&amp;O27&amp;", "&amp;P27&amp;" }"&amp;", "&amp;" { "&amp;Q27&amp;", "&amp;R27&amp;", "&amp;S27&amp;", "&amp;T27&amp;" }"&amp;", "&amp;" { "&amp;U27&amp;", "&amp;V27&amp;", "&amp;W27&amp;", "&amp;X27&amp;" }"&amp;", "&amp;" { "&amp;Y27&amp;", "&amp;Z27&amp;", "&amp;AA27&amp;", "&amp;AB27&amp;" }"&amp;" }"&amp;" } },")</f>
         <v/>
       </c>
     </row>
@@ -6789,7 +6784,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Copy column A (values shown) from BEGIN through END into QuestionnaireConfig.h. Includes NUM_QUESTIONS and QUESTIONS[]. Skip empty lines in the array. Row count = filled Artwork cells on Questions sheet.</t>
+          <t>Copy column A from BEGIN through END into QuestionnaireConfig.h. Lines pull live from Questions (scores, screen, step). Skip blank array lines. NUM_QUESTIONS = COUNTA(Artwork). Recalculate the sheet after edits (F9 in Excel).</t>
         </is>
       </c>
     </row>

</xml_diff>